<commit_message>
fix: harden complex-document retrieval and citation validation
</commit_message>
<xml_diff>
--- a/backend/tests/golden/corpus/xlsx_clean.xlsx
+++ b/backend/tests/golden/corpus/xlsx_clean.xlsx
@@ -11,94 +11,94 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetData>
     <row r="1">
-      <c r="@1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>指标</t>
         </is>
       </c>
-      <c r="A1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>2023年</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>2024年</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>同比</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="@2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>营业收入</t>
         </is>
       </c>
-      <c r="A2">
+      <c r="B2">
         <v>30240</v>
       </c>
-      <c r="B2">
+      <c r="C2">
         <v>33500</v>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>+10.8%</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="@3" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>净利润</t>
         </is>
       </c>
-      <c r="A3">
+      <c r="B3">
         <v>2180</v>
       </c>
-      <c r="B3">
+      <c r="C3">
         <v>2460</v>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>+12.8%</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="@4" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>毛利率</t>
         </is>
       </c>
-      <c r="A4" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>24.1%</t>
         </is>
       </c>
-      <c r="B4"/>
-      <c r="C4" t="inlineStr">
+      <c r="C4"/>
+      <c r="D4" t="inlineStr">
         <is>
           <t>+0.9pp</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="@5" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>研发投入</t>
         </is>
       </c>
-      <c r="A5">
+      <c r="B5">
         <v>1520</v>
       </c>
-      <c r="B5">
+      <c r="C5">
         <v>1810</v>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>+19.1%</t>
         </is>

</xml_diff>